<commit_message>
fixed readme, added instruction for table fill in, in the gui, and renamed some of the readmes
</commit_message>
<xml_diff>
--- a/documentation/testing/plannerTestingGraphs.xlsx
+++ b/documentation/testing/plannerTestingGraphs.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="20">
   <si>
     <t xml:space="preserve">data brando</t>
   </si>
@@ -89,7 +89,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -113,23 +113,20 @@
       <family val="0"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="13"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -176,7 +173,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -185,23 +182,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -290,11 +275,17 @@
           <a:p>
             <a:pPr>
               <a:defRPr b="0" sz="1300" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:latin typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
             <a:r>
               <a:rPr b="0" sz="1300" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:latin typeface="Arial"/>
               </a:rPr>
               <a:t>Tempo di esecuzione totale vs. difficoltà</a:t>
@@ -356,11 +347,15 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="r"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -441,11 +436,15 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="r"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -490,11 +489,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="80409623"/>
-        <c:axId val="56421508"/>
+        <c:axId val="75402765"/>
+        <c:axId val="49106136"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="80409623"/>
+        <c:axId val="75402765"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -508,11 +507,17 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="900" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
                   <a:rPr b="0" sz="900" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:rPr>
                   <a:t>difficoltà</a:t>
@@ -528,7 +533,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -545,12 +550,15 @@
           <a:p>
             <a:pPr>
               <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:latin typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="56421508"/>
+        <c:crossAx val="49106136"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -558,7 +566,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="56421508"/>
+        <c:axId val="49106136"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -581,11 +589,17 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="900" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
                   <a:rPr b="0" sz="900" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:rPr>
                   <a:t>Tempo di esecuzione medio</a:t>
@@ -601,7 +615,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -618,12 +632,15 @@
           <a:p>
             <a:pPr>
               <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:latin typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="80409623"/>
+        <c:crossAx val="75402765"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -651,6 +668,9 @@
         <a:p>
           <a:pPr>
             <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
               <a:latin typeface="Arial"/>
             </a:defRPr>
           </a:pPr>
@@ -684,11 +704,17 @@
           <a:p>
             <a:pPr>
               <a:defRPr b="0" sz="1300" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:latin typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
             <a:r>
               <a:rPr b="0" sz="1300" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:latin typeface="Arial"/>
               </a:rPr>
               <a:t>Grounding vs Planning Tiime</a:t>
@@ -740,11 +766,15 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="ctr"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -851,11 +881,15 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="ctr"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -962,11 +996,15 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="ctr"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -1070,11 +1108,15 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="ctr"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -1150,11 +1192,11 @@
         </c:ser>
         <c:gapWidth val="50"/>
         <c:overlap val="100"/>
-        <c:axId val="61452460"/>
-        <c:axId val="9151825"/>
+        <c:axId val="28837638"/>
+        <c:axId val="90736808"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="61452460"/>
+        <c:axId val="28837638"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1168,11 +1210,17 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="900" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
                   <a:rPr b="0" sz="900" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:rPr>
                   <a:t>Difficoltà</a:t>
@@ -1188,7 +1236,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1205,12 +1253,15 @@
           <a:p>
             <a:pPr>
               <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:latin typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="9151825"/>
+        <c:crossAx val="90736808"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1218,7 +1269,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="9151825"/>
+        <c:axId val="90736808"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1241,11 +1292,17 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="900" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
                   <a:rPr b="0" sz="900" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:rPr>
                   <a:t>Tempo [ms]</a:t>
@@ -1261,7 +1318,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1278,12 +1335,15 @@
           <a:p>
             <a:pPr>
               <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:latin typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61452460"/>
+        <c:crossAx val="28837638"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1311,6 +1371,9 @@
         <a:p>
           <a:pPr>
             <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
               <a:latin typeface="Arial"/>
             </a:defRPr>
           </a:pPr>
@@ -1336,15 +1399,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>923040</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>141120</xdr:rowOff>
+      <xdr:colOff>226080</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>67320</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>138240</xdr:colOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>784440</xdr:colOff>
       <xdr:row>41</xdr:row>
-      <xdr:rowOff>19080</xdr:rowOff>
+      <xdr:rowOff>71280</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1352,8 +1415,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="7144920" y="1284120"/>
-        <a:ext cx="11637000" cy="6545520"/>
+        <a:off x="6447960" y="3877200"/>
+        <a:ext cx="7119720" cy="4004640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1371,10 +1434,10 @@
       <xdr:rowOff>57600</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>471960</xdr:colOff>
-      <xdr:row>88</xdr:row>
-      <xdr:rowOff>138960</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>669960</xdr:colOff>
+      <xdr:row>75</xdr:row>
+      <xdr:rowOff>107640</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1383,7 +1446,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="6251040" y="10344600"/>
-        <a:ext cx="11660400" cy="6558480"/>
+        <a:ext cx="7202160" cy="4050720"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1576,20 +1639,20 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:L53"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="23.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="19.1"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="23.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="23.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="20.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="25.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="23.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="19.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="23.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="22.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="23.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="20.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="25.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="23.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="19.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="23.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="22.58"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1605,7 +1668,7 @@
       <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
       <c r="G1" s="2" t="s">
@@ -1634,31 +1697,31 @@
       <c r="B2" s="1" t="n">
         <v>533</v>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="C2" s="2" t="n">
         <v>497</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D2" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="F2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G2" s="0" t="n">
+      <c r="G2" s="1" t="n">
         <v>508.666666666667</v>
       </c>
-      <c r="H2" s="0" t="n">
+      <c r="H2" s="1" t="n">
         <v>469.333333333333</v>
       </c>
-      <c r="I2" s="0" t="n">
+      <c r="I2" s="1" t="n">
         <v>39.3333333333333</v>
       </c>
       <c r="J2" s="1" t="n">
         <v>1528.66666666667</v>
       </c>
-      <c r="K2" s="0" t="n">
+      <c r="K2" s="1" t="n">
         <v>1421</v>
       </c>
-      <c r="L2" s="0" t="n">
+      <c r="L2" s="1" t="n">
         <v>107.666666666667</v>
       </c>
     </row>
@@ -1666,10 +1729,10 @@
       <c r="B3" s="1" t="n">
         <v>485</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" s="2" t="n">
         <v>446</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D3" s="2" t="n">
         <v>39</v>
       </c>
       <c r="F3" s="2" t="n">
@@ -1678,19 +1741,19 @@
       <c r="G3" s="1" t="n">
         <v>877.333333333333</v>
       </c>
-      <c r="H3" s="0" t="n">
+      <c r="H3" s="1" t="n">
         <v>754.666666666667</v>
       </c>
-      <c r="I3" s="0" t="n">
+      <c r="I3" s="1" t="n">
         <v>122.666666666667</v>
       </c>
-      <c r="J3" s="0" t="n">
+      <c r="J3" s="1" t="n">
         <v>2640</v>
       </c>
-      <c r="K3" s="0" t="n">
+      <c r="K3" s="1" t="n">
         <v>2196</v>
       </c>
-      <c r="L3" s="0" t="n">
+      <c r="L3" s="1" t="n">
         <v>444</v>
       </c>
     </row>
@@ -1698,31 +1761,31 @@
       <c r="B4" s="1" t="n">
         <v>508</v>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C4" s="2" t="n">
         <v>465</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="D4" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="F4" s="2" t="n">
         <v>3</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>2951</v>
       </c>
-      <c r="H4" s="0" t="n">
+      <c r="H4" s="1" t="n">
         <v>2158.33333333333</v>
       </c>
-      <c r="I4" s="0" t="n">
+      <c r="I4" s="1" t="n">
         <v>792.666666666667</v>
       </c>
       <c r="J4" s="1" t="n">
         <v>8464.33333333333</v>
       </c>
-      <c r="K4" s="0" t="n">
+      <c r="K4" s="1" t="n">
         <v>6838.66666666667</v>
       </c>
-      <c r="L4" s="0" t="n">
+      <c r="L4" s="1" t="n">
         <v>1625.66666666667</v>
       </c>
     </row>
@@ -1748,19 +1811,19 @@
       <c r="G5" s="1" t="n">
         <v>7535.33333333333</v>
       </c>
-      <c r="H5" s="0" t="n">
+      <c r="H5" s="1" t="n">
         <v>3898.66666666667</v>
       </c>
-      <c r="I5" s="0" t="n">
+      <c r="I5" s="1" t="n">
         <v>3636.66666666667</v>
       </c>
       <c r="J5" s="1" t="n">
         <v>16229.3333333333</v>
       </c>
-      <c r="K5" s="0" t="n">
+      <c r="K5" s="1" t="n">
         <v>11226.3333333333</v>
       </c>
-      <c r="L5" s="0" t="n">
+      <c r="L5" s="1" t="n">
         <v>5003</v>
       </c>
     </row>
@@ -1771,31 +1834,28 @@
       <c r="B6" s="1" t="n">
         <v>866</v>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C6" s="2" t="n">
         <v>745</v>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="D6" s="2" t="n">
         <v>121</v>
       </c>
-      <c r="F6" s="3" t="n">
+      <c r="F6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G6" s="0" t="n">
+      <c r="G6" s="1" t="n">
         <v>7947</v>
       </c>
-      <c r="H6" s="0" t="n">
+      <c r="H6" s="1" t="n">
         <v>5387</v>
       </c>
-      <c r="I6" s="0" t="n">
+      <c r="I6" s="1" t="n">
         <v>2560</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="K6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="K6" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="L6" s="4" t="s">
+      <c r="L6" s="2" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1803,26 +1863,23 @@
       <c r="B7" s="2" t="n">
         <v>877</v>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C7" s="2" t="n">
         <v>757</v>
       </c>
-      <c r="D7" s="3" t="n">
+      <c r="D7" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="1" t="n">
         <v>889</v>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C8" s="2" t="n">
         <v>762</v>
       </c>
-      <c r="D8" s="3" t="n">
+      <c r="D8" s="2" t="n">
         <v>127</v>
       </c>
-      <c r="F8" s="1"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
@@ -1840,7 +1897,6 @@
         <f aca="false">AVERAGE(D6:D8)</f>
         <v>122.666666666667</v>
       </c>
-      <c r="F9" s="1"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
@@ -1849,10 +1905,10 @@
       <c r="B10" s="1" t="n">
         <v>3022</v>
       </c>
-      <c r="C10" s="3" t="n">
+      <c r="C10" s="2" t="n">
         <v>2221</v>
       </c>
-      <c r="D10" s="3" t="n">
+      <c r="D10" s="2" t="n">
         <v>801</v>
       </c>
     </row>
@@ -1860,25 +1916,23 @@
       <c r="B11" s="1" t="n">
         <v>2930</v>
       </c>
-      <c r="C11" s="3" t="n">
+      <c r="C11" s="2" t="n">
         <v>2128</v>
       </c>
-      <c r="D11" s="3" t="n">
+      <c r="D11" s="2" t="n">
         <v>802</v>
       </c>
-      <c r="F11" s="1"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="1" t="n">
         <v>2901</v>
       </c>
-      <c r="C12" s="3" t="n">
+      <c r="C12" s="2" t="n">
         <v>2126</v>
       </c>
-      <c r="D12" s="3" t="n">
+      <c r="D12" s="2" t="n">
         <v>775</v>
       </c>
-      <c r="F12" s="1"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
@@ -1896,7 +1950,6 @@
         <f aca="false">AVERAGE(D10:D12)</f>
         <v>792.666666666667</v>
       </c>
-      <c r="F13" s="1"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
@@ -1905,10 +1958,10 @@
       <c r="B14" s="1" t="n">
         <v>7958</v>
       </c>
-      <c r="C14" s="3" t="n">
+      <c r="C14" s="2" t="n">
         <v>4306</v>
       </c>
-      <c r="D14" s="3" t="n">
+      <c r="D14" s="2" t="n">
         <v>3652</v>
       </c>
     </row>
@@ -1916,27 +1969,23 @@
       <c r="B15" s="1" t="n">
         <v>7278</v>
       </c>
-      <c r="C15" s="3" t="n">
+      <c r="C15" s="2" t="n">
         <v>3719</v>
       </c>
-      <c r="D15" s="3" t="n">
+      <c r="D15" s="2" t="n">
         <v>3559</v>
       </c>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="1" t="n">
         <v>7370</v>
       </c>
-      <c r="C16" s="3" t="n">
+      <c r="C16" s="2" t="n">
         <v>3671</v>
       </c>
-      <c r="D16" s="3" t="n">
+      <c r="D16" s="2" t="n">
         <v>3699</v>
       </c>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
@@ -1954,8 +2003,6 @@
         <f aca="false">AVERAGE(D14:D16)</f>
         <v>3636.66666666667</v>
       </c>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
@@ -1964,39 +2011,37 @@
       <c r="B18" s="1" t="n">
         <v>7801</v>
       </c>
-      <c r="C18" s="3" t="n">
+      <c r="C18" s="2" t="n">
         <v>5198</v>
       </c>
-      <c r="D18" s="3" t="n">
+      <c r="D18" s="2" t="n">
         <v>2603</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0"/>
       <c r="B19" s="1" t="n">
         <v>7939</v>
       </c>
-      <c r="C19" s="3" t="n">
+      <c r="C19" s="2" t="n">
         <v>5473</v>
       </c>
-      <c r="D19" s="3" t="n">
+      <c r="D19" s="2" t="n">
         <v>2466</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0"/>
       <c r="B20" s="1" t="n">
         <v>8101</v>
       </c>
-      <c r="C20" s="3" t="n">
+      <c r="C20" s="2" t="n">
         <v>5490</v>
       </c>
-      <c r="D20" s="3" t="n">
+      <c r="D20" s="2" t="n">
         <v>2611</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B21" s="1" t="n">
@@ -2012,12 +2057,6 @@
         <v>2560</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0"/>
-      <c r="B22" s="0"/>
-      <c r="C22" s="0"/>
-      <c r="D22" s="0"/>
-    </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
         <v>18</v>
@@ -2027,35 +2066,35 @@
       <c r="A24" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B24" s="5" t="n">
+      <c r="B24" s="2" t="n">
         <v>1455</v>
       </c>
-      <c r="C24" s="5" t="n">
+      <c r="C24" s="2" t="n">
         <v>1345</v>
       </c>
-      <c r="D24" s="5" t="n">
+      <c r="D24" s="2" t="n">
         <v>110</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="5" t="n">
+      <c r="B25" s="2" t="n">
         <v>1577</v>
       </c>
-      <c r="C25" s="5" t="n">
+      <c r="C25" s="2" t="n">
         <v>1469</v>
       </c>
-      <c r="D25" s="5" t="n">
+      <c r="D25" s="2" t="n">
         <v>108</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="5" t="n">
+      <c r="B26" s="2" t="n">
         <v>1554</v>
       </c>
-      <c r="C26" s="5" t="n">
+      <c r="C26" s="2" t="n">
         <v>1449</v>
       </c>
-      <c r="D26" s="5" t="n">
+      <c r="D26" s="2" t="n">
         <v>105</v>
       </c>
     </row>
@@ -2080,35 +2119,35 @@
       <c r="A28" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B28" s="5" t="n">
+      <c r="B28" s="2" t="n">
         <v>2745</v>
       </c>
-      <c r="C28" s="5" t="n">
+      <c r="C28" s="2" t="n">
         <v>2252</v>
       </c>
-      <c r="D28" s="5" t="n">
+      <c r="D28" s="2" t="n">
         <v>493</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="5" t="n">
+      <c r="B29" s="2" t="n">
         <v>2544</v>
       </c>
-      <c r="C29" s="5" t="n">
+      <c r="C29" s="2" t="n">
         <v>2118</v>
       </c>
-      <c r="D29" s="5" t="n">
+      <c r="D29" s="2" t="n">
         <v>426</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="5" t="n">
+      <c r="B30" s="2" t="n">
         <v>2631</v>
       </c>
-      <c r="C30" s="5" t="n">
+      <c r="C30" s="2" t="n">
         <v>2218</v>
       </c>
-      <c r="D30" s="5" t="n">
+      <c r="D30" s="2" t="n">
         <v>413</v>
       </c>
     </row>
@@ -2133,35 +2172,35 @@
       <c r="A32" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B32" s="5" t="n">
+      <c r="B32" s="2" t="n">
         <v>8470</v>
       </c>
-      <c r="C32" s="5" t="n">
+      <c r="C32" s="2" t="n">
         <v>6861</v>
       </c>
-      <c r="D32" s="5" t="n">
+      <c r="D32" s="2" t="n">
         <v>1609</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="5" t="n">
+      <c r="B33" s="2" t="n">
         <v>8220</v>
       </c>
-      <c r="C33" s="5" t="n">
+      <c r="C33" s="2" t="n">
         <v>6561</v>
       </c>
-      <c r="D33" s="5" t="n">
+      <c r="D33" s="2" t="n">
         <v>1659</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="5" t="n">
+      <c r="B34" s="2" t="n">
         <v>8703</v>
       </c>
-      <c r="C34" s="5" t="n">
+      <c r="C34" s="2" t="n">
         <v>7094</v>
       </c>
-      <c r="D34" s="5" t="n">
+      <c r="D34" s="2" t="n">
         <v>1609</v>
       </c>
     </row>
@@ -2186,35 +2225,35 @@
       <c r="A36" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B36" s="5" t="n">
+      <c r="B36" s="2" t="n">
         <v>16722</v>
       </c>
-      <c r="C36" s="5" t="n">
+      <c r="C36" s="2" t="n">
         <v>11440</v>
       </c>
-      <c r="D36" s="5" t="n">
+      <c r="D36" s="2" t="n">
         <v>5282</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="5" t="n">
+      <c r="B37" s="2" t="n">
         <v>16253</v>
       </c>
-      <c r="C37" s="5" t="n">
+      <c r="C37" s="2" t="n">
         <v>11080</v>
       </c>
-      <c r="D37" s="5" t="n">
+      <c r="D37" s="2" t="n">
         <v>5173</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="5" t="n">
+      <c r="B38" s="2" t="n">
         <v>15713</v>
       </c>
-      <c r="C38" s="5" t="n">
+      <c r="C38" s="2" t="n">
         <v>11159</v>
       </c>
-      <c r="D38" s="5" t="n">
+      <c r="D38" s="2" t="n">
         <v>4554</v>
       </c>
     </row>
@@ -2239,34 +2278,30 @@
       <c r="A40" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B40" s="6" t="s">
+      <c r="B40" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C40" s="6" t="s">
+      <c r="C40" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D40" s="6" t="s">
+      <c r="D40" s="3" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="4"/>
-      <c r="B41" s="6" t="s">
+      <c r="A41" s="2"/>
+      <c r="B41" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C41" s="6" t="s">
+      <c r="C41" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D41" s="6" t="s">
+      <c r="D41" s="3" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="0"/>
-      <c r="B43" s="0"/>
-      <c r="C43" s="0"/>
-      <c r="D43" s="0"/>
-      <c r="F43" s="3" t="s">
+      <c r="F43" s="2" t="s">
         <v>4</v>
       </c>
       <c r="G43" s="2" t="s">
@@ -2283,202 +2318,108 @@
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="0"/>
-      <c r="B44" s="0"/>
-      <c r="C44" s="0"/>
-      <c r="D44" s="0"/>
-      <c r="F44" s="3" t="n">
+      <c r="F44" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G44" s="0" t="n">
+      <c r="G44" s="1" t="n">
         <v>469.333333333333</v>
       </c>
-      <c r="H44" s="0" t="n">
+      <c r="H44" s="1" t="n">
         <v>39.3333333333333</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="0"/>
-      <c r="B45" s="0"/>
-      <c r="C45" s="0"/>
-      <c r="D45" s="0"/>
-      <c r="F45" s="0" t="n">
+      <c r="F45" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I45" s="0" t="n">
+      <c r="I45" s="1" t="n">
         <v>1421</v>
       </c>
-      <c r="J45" s="0" t="n">
+      <c r="J45" s="1" t="n">
         <v>107.666666666667</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="0"/>
-      <c r="B46" s="0"/>
-      <c r="C46" s="0"/>
-      <c r="D46" s="0"/>
       <c r="F46" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G46" s="0" t="n">
+      <c r="G46" s="1" t="n">
         <v>754.666666666667</v>
       </c>
-      <c r="H46" s="0" t="n">
+      <c r="H46" s="1" t="n">
         <v>122.666666666667</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="0"/>
-      <c r="B47" s="0"/>
-      <c r="C47" s="0"/>
-      <c r="D47" s="0"/>
-      <c r="F47" s="0" t="n">
+      <c r="F47" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I47" s="0" t="n">
+      <c r="I47" s="1" t="n">
         <v>2196</v>
       </c>
-      <c r="J47" s="0" t="n">
+      <c r="J47" s="1" t="n">
         <v>444</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="0"/>
-      <c r="B48" s="0"/>
-      <c r="C48" s="0"/>
-      <c r="D48" s="0"/>
-      <c r="F48" s="3" t="n">
+      <c r="F48" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G48" s="0" t="n">
+      <c r="G48" s="1" t="n">
         <v>2158.33333333333</v>
       </c>
-      <c r="H48" s="0" t="n">
+      <c r="H48" s="1" t="n">
         <v>792.666666666667</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="0"/>
-      <c r="B49" s="0"/>
-      <c r="C49" s="0"/>
-      <c r="D49" s="0"/>
-      <c r="F49" s="0" t="n">
+      <c r="F49" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="I49" s="0" t="n">
+      <c r="I49" s="1" t="n">
         <v>6838.66666666667</v>
       </c>
-      <c r="J49" s="0" t="n">
+      <c r="J49" s="1" t="n">
         <v>1625.66666666667</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="0"/>
-      <c r="B50" s="0"/>
-      <c r="C50" s="0"/>
-      <c r="D50" s="0"/>
       <c r="F50" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G50" s="0" t="n">
+      <c r="G50" s="1" t="n">
         <v>3898.66666666667</v>
       </c>
-      <c r="H50" s="0" t="n">
+      <c r="H50" s="1" t="n">
         <v>3636.66666666667</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="0"/>
-      <c r="B51" s="0"/>
-      <c r="C51" s="0"/>
-      <c r="D51" s="0"/>
-      <c r="F51" s="0" t="n">
+      <c r="F51" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="I51" s="0" t="n">
+      <c r="I51" s="1" t="n">
         <v>11226.3333333333</v>
       </c>
-      <c r="J51" s="0" t="n">
+      <c r="J51" s="1" t="n">
         <v>5003</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="0"/>
-      <c r="B52" s="0"/>
-      <c r="C52" s="0"/>
-      <c r="D52" s="0"/>
-      <c r="F52" s="3" t="n">
+      <c r="F52" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G52" s="0" t="n">
+      <c r="G52" s="1" t="n">
         <v>5387</v>
       </c>
-      <c r="H52" s="0" t="n">
+      <c r="H52" s="1" t="n">
         <v>2560</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="0"/>
-      <c r="B53" s="0"/>
-      <c r="C53" s="0"/>
-      <c r="D53" s="0"/>
-      <c r="F53" s="0" t="n">
+      <c r="F53" s="1" t="n">
         <v>5</v>
       </c>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="0"/>
-      <c r="B54" s="0"/>
-      <c r="C54" s="0"/>
-      <c r="D54" s="0"/>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="0"/>
-      <c r="B55" s="0"/>
-      <c r="C55" s="0"/>
-      <c r="D55" s="0"/>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="0"/>
-      <c r="B56" s="0"/>
-      <c r="C56" s="0"/>
-      <c r="D56" s="0"/>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="0"/>
-      <c r="B57" s="0"/>
-      <c r="C57" s="0"/>
-      <c r="D57" s="0"/>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="0"/>
-      <c r="B58" s="0"/>
-      <c r="C58" s="0"/>
-      <c r="D58" s="0"/>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="0"/>
-      <c r="B59" s="0"/>
-      <c r="C59" s="0"/>
-      <c r="D59" s="0"/>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="0"/>
-      <c r="B60" s="0"/>
-      <c r="C60" s="0"/>
-      <c r="D60" s="0"/>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="0"/>
-      <c r="B61" s="0"/>
-      <c r="C61" s="0"/>
-      <c r="D61" s="0"/>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="0"/>
-      <c r="B62" s="0"/>
-      <c r="C62" s="0"/>
-      <c r="D62" s="0"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>